<commit_message>
Generate facility templates from master layout
</commit_message>
<xml_diff>
--- a/backend/src/data/order_form_master_templates/master_layout_template.xlsx
+++ b/backend/src/data/order_form_master_templates/master_layout_template.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,11 +31,6 @@
     <font>
       <name val="Yu Gothic"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Yu Gothic"/>
-      <b val="1"/>
-      <sz val="14"/>
     </font>
     <font>
       <name val="Yu Gothic"/>
@@ -583,24 +578,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -624,27 +613,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -661,7 +650,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -680,7 +669,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -699,7 +688,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -713,9 +702,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1157,1385 +1143,1373 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="3" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>【発　注　連　絡　表】</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>FAX送信先：050-3092-0899</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>施設名ご記入お願いします。</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>締切日　月　日まで</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="7" t="n"/>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="10" t="inlineStr">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>※ご希望メニューに食数をご記入ください。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="11" t="n"/>
-      <c r="B5" s="12" t="n"/>
-      <c r="C5" s="12" t="n"/>
-      <c r="D5" s="12" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="n"/>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="n"/>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>※禁止食材は禁食欄に「食事種類と食数」ご記入ください。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
     </row>
     <row r="7" ht="23" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>日　付</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>区　分</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>献立</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="18" t="n"/>
-      <c r="N7" s="16" t="n"/>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
+      <c r="M7" s="16" t="n"/>
+      <c r="N7" s="14" t="n"/>
     </row>
     <row r="8" ht="23" customHeight="1">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="20" t="n"/>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="20" t="n"/>
-      <c r="M8" s="20" t="n"/>
-      <c r="N8" s="21" t="n"/>
+      <c r="A8" s="17" t="n"/>
+      <c r="B8" s="18" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="18" t="n"/>
+      <c r="M8" s="18" t="n"/>
+      <c r="N8" s="19" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D9" s="25" t="n"/>
-      <c r="E9" s="26" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="27" t="n"/>
-      <c r="I9" s="27" t="n"/>
-      <c r="J9" s="27" t="n"/>
-      <c r="K9" s="27" t="n"/>
-      <c r="L9" s="27" t="n"/>
-      <c r="M9" s="27" t="n"/>
-      <c r="N9" s="28" t="n"/>
+      <c r="D9" s="23" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="25" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="25" t="n"/>
+      <c r="L9" s="25" t="n"/>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="26" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="29" t="n"/>
-      <c r="B10" s="30" t="n"/>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="A10" s="27" t="n"/>
+      <c r="B10" s="28" t="n"/>
+      <c r="C10" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="34" t="n"/>
-      <c r="G10" s="34" t="n"/>
-      <c r="H10" s="34" t="n"/>
-      <c r="I10" s="34" t="n"/>
-      <c r="J10" s="34" t="n"/>
-      <c r="K10" s="34" t="n"/>
-      <c r="L10" s="34" t="n"/>
-      <c r="M10" s="34" t="n"/>
-      <c r="N10" s="35" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
+      <c r="H10" s="32" t="n"/>
+      <c r="I10" s="32" t="n"/>
+      <c r="J10" s="32" t="n"/>
+      <c r="K10" s="32" t="n"/>
+      <c r="L10" s="32" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="33" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="36" t="n"/>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="A11" s="34" t="n"/>
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C11" s="38" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D11" s="39" t="n"/>
-      <c r="E11" s="40" t="n"/>
-      <c r="F11" s="41" t="n"/>
-      <c r="G11" s="41" t="n"/>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="41" t="n"/>
-      <c r="J11" s="41" t="n"/>
-      <c r="K11" s="41" t="n"/>
-      <c r="L11" s="41" t="n"/>
-      <c r="M11" s="41" t="n"/>
-      <c r="N11" s="42" t="n"/>
+      <c r="D11" s="37" t="n"/>
+      <c r="E11" s="38" t="n"/>
+      <c r="F11" s="39" t="n"/>
+      <c r="G11" s="39" t="n"/>
+      <c r="H11" s="39" t="n"/>
+      <c r="I11" s="39" t="n"/>
+      <c r="J11" s="39" t="n"/>
+      <c r="K11" s="39" t="n"/>
+      <c r="L11" s="39" t="n"/>
+      <c r="M11" s="39" t="n"/>
+      <c r="N11" s="40" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="29" t="n"/>
-      <c r="B12" s="30" t="n"/>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="A12" s="27" t="n"/>
+      <c r="B12" s="28" t="n"/>
+      <c r="C12" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D12" s="32" t="n"/>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="34" t="n"/>
-      <c r="G12" s="34" t="n"/>
-      <c r="H12" s="34" t="n"/>
-      <c r="I12" s="34" t="n"/>
-      <c r="J12" s="34" t="n"/>
-      <c r="K12" s="34" t="n"/>
-      <c r="L12" s="34" t="n"/>
-      <c r="M12" s="34" t="n"/>
-      <c r="N12" s="35" t="n"/>
+      <c r="D12" s="30" t="n"/>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="32" t="n"/>
+      <c r="G12" s="32" t="n"/>
+      <c r="H12" s="32" t="n"/>
+      <c r="I12" s="32" t="n"/>
+      <c r="J12" s="32" t="n"/>
+      <c r="K12" s="32" t="n"/>
+      <c r="L12" s="32" t="n"/>
+      <c r="M12" s="32" t="n"/>
+      <c r="N12" s="33" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="43" t="n"/>
-      <c r="B13" s="30" t="n"/>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="A13" s="41" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D13" s="32" t="n"/>
-      <c r="E13" s="33" t="n"/>
-      <c r="F13" s="34" t="n"/>
-      <c r="G13" s="34" t="n"/>
-      <c r="H13" s="34" t="n"/>
-      <c r="I13" s="34" t="n"/>
-      <c r="J13" s="34" t="n"/>
-      <c r="K13" s="34" t="n"/>
-      <c r="L13" s="34" t="n"/>
-      <c r="M13" s="34" t="n"/>
-      <c r="N13" s="35" t="n"/>
+      <c r="D13" s="30" t="n"/>
+      <c r="E13" s="31" t="n"/>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="32" t="n"/>
+      <c r="H13" s="32" t="n"/>
+      <c r="I13" s="32" t="n"/>
+      <c r="J13" s="32" t="n"/>
+      <c r="K13" s="32" t="n"/>
+      <c r="L13" s="32" t="n"/>
+      <c r="M13" s="32" t="n"/>
+      <c r="N13" s="33" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="44" t="n"/>
-      <c r="B14" s="37" t="inlineStr">
+      <c r="A14" s="42" t="n"/>
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="C14" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D14" s="39" t="n"/>
-      <c r="E14" s="40" t="n"/>
-      <c r="F14" s="41" t="n"/>
-      <c r="G14" s="41" t="n"/>
-      <c r="H14" s="41" t="n"/>
-      <c r="I14" s="41" t="n"/>
-      <c r="J14" s="41" t="n"/>
-      <c r="K14" s="41" t="n"/>
-      <c r="L14" s="41" t="n"/>
-      <c r="M14" s="41" t="n"/>
-      <c r="N14" s="42" t="n"/>
+      <c r="D14" s="37" t="n"/>
+      <c r="E14" s="38" t="n"/>
+      <c r="F14" s="39" t="n"/>
+      <c r="G14" s="39" t="n"/>
+      <c r="H14" s="39" t="n"/>
+      <c r="I14" s="39" t="n"/>
+      <c r="J14" s="39" t="n"/>
+      <c r="K14" s="39" t="n"/>
+      <c r="L14" s="39" t="n"/>
+      <c r="M14" s="39" t="n"/>
+      <c r="N14" s="40" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="29" t="n"/>
-      <c r="B15" s="30" t="n"/>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="A15" s="27" t="n"/>
+      <c r="B15" s="28" t="n"/>
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D15" s="32" t="n"/>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="34" t="n"/>
-      <c r="G15" s="34" t="n"/>
-      <c r="H15" s="34" t="n"/>
-      <c r="I15" s="34" t="n"/>
-      <c r="J15" s="34" t="n"/>
-      <c r="K15" s="34" t="n"/>
-      <c r="L15" s="34" t="n"/>
-      <c r="M15" s="34" t="n"/>
-      <c r="N15" s="35" t="n"/>
+      <c r="D15" s="30" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="32" t="n"/>
+      <c r="G15" s="32" t="n"/>
+      <c r="H15" s="32" t="n"/>
+      <c r="I15" s="32" t="n"/>
+      <c r="J15" s="32" t="n"/>
+      <c r="K15" s="32" t="n"/>
+      <c r="L15" s="32" t="n"/>
+      <c r="M15" s="32" t="n"/>
+      <c r="N15" s="33" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="46" t="n"/>
-      <c r="C16" s="47" t="inlineStr">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="n"/>
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D16" s="48" t="n"/>
-      <c r="E16" s="49" t="n"/>
-      <c r="F16" s="50" t="n"/>
-      <c r="G16" s="50" t="n"/>
-      <c r="H16" s="50" t="n"/>
-      <c r="I16" s="50" t="n"/>
-      <c r="J16" s="50" t="n"/>
-      <c r="K16" s="50" t="n"/>
-      <c r="L16" s="50" t="n"/>
-      <c r="M16" s="50" t="n"/>
-      <c r="N16" s="51" t="n"/>
+      <c r="D16" s="46" t="n"/>
+      <c r="E16" s="47" t="n"/>
+      <c r="F16" s="48" t="n"/>
+      <c r="G16" s="48" t="n"/>
+      <c r="H16" s="48" t="n"/>
+      <c r="I16" s="48" t="n"/>
+      <c r="J16" s="48" t="n"/>
+      <c r="K16" s="48" t="n"/>
+      <c r="L16" s="48" t="n"/>
+      <c r="M16" s="48" t="n"/>
+      <c r="N16" s="49" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D17" s="25" t="n"/>
-      <c r="E17" s="26" t="n"/>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
-      <c r="H17" s="27" t="n"/>
-      <c r="I17" s="27" t="n"/>
-      <c r="J17" s="27" t="n"/>
-      <c r="K17" s="27" t="n"/>
-      <c r="L17" s="27" t="n"/>
-      <c r="M17" s="27" t="n"/>
-      <c r="N17" s="28" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
+      <c r="J17" s="25" t="n"/>
+      <c r="K17" s="25" t="n"/>
+      <c r="L17" s="25" t="n"/>
+      <c r="M17" s="25" t="n"/>
+      <c r="N17" s="26" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="29" t="n"/>
-      <c r="B18" s="30" t="n"/>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="A18" s="27" t="n"/>
+      <c r="B18" s="28" t="n"/>
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="33" t="n"/>
-      <c r="F18" s="34" t="n"/>
-      <c r="G18" s="34" t="n"/>
-      <c r="H18" s="34" t="n"/>
-      <c r="I18" s="34" t="n"/>
-      <c r="J18" s="34" t="n"/>
-      <c r="K18" s="34" t="n"/>
-      <c r="L18" s="34" t="n"/>
-      <c r="M18" s="34" t="n"/>
-      <c r="N18" s="35" t="n"/>
+      <c r="D18" s="30" t="n"/>
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="32" t="n"/>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="32" t="n"/>
+      <c r="J18" s="32" t="n"/>
+      <c r="K18" s="32" t="n"/>
+      <c r="L18" s="32" t="n"/>
+      <c r="M18" s="32" t="n"/>
+      <c r="N18" s="33" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="36" t="n"/>
-      <c r="B19" s="37" t="inlineStr">
+      <c r="A19" s="34" t="n"/>
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C19" s="38" t="inlineStr">
+      <c r="C19" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D19" s="39" t="n"/>
-      <c r="E19" s="40" t="n"/>
-      <c r="F19" s="41" t="n"/>
-      <c r="G19" s="41" t="n"/>
-      <c r="H19" s="41" t="n"/>
-      <c r="I19" s="41" t="n"/>
-      <c r="J19" s="41" t="n"/>
-      <c r="K19" s="41" t="n"/>
-      <c r="L19" s="41" t="n"/>
-      <c r="M19" s="41" t="n"/>
-      <c r="N19" s="42" t="n"/>
+      <c r="D19" s="37" t="n"/>
+      <c r="E19" s="38" t="n"/>
+      <c r="F19" s="39" t="n"/>
+      <c r="G19" s="39" t="n"/>
+      <c r="H19" s="39" t="n"/>
+      <c r="I19" s="39" t="n"/>
+      <c r="J19" s="39" t="n"/>
+      <c r="K19" s="39" t="n"/>
+      <c r="L19" s="39" t="n"/>
+      <c r="M19" s="39" t="n"/>
+      <c r="N19" s="40" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="29" t="n"/>
-      <c r="B20" s="30" t="n"/>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="A20" s="27" t="n"/>
+      <c r="B20" s="28" t="n"/>
+      <c r="C20" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D20" s="32" t="n"/>
-      <c r="E20" s="33" t="n"/>
-      <c r="F20" s="34" t="n"/>
-      <c r="G20" s="34" t="n"/>
-      <c r="H20" s="34" t="n"/>
-      <c r="I20" s="34" t="n"/>
-      <c r="J20" s="34" t="n"/>
-      <c r="K20" s="34" t="n"/>
-      <c r="L20" s="34" t="n"/>
-      <c r="M20" s="34" t="n"/>
-      <c r="N20" s="35" t="n"/>
+      <c r="D20" s="30" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="32" t="n"/>
+      <c r="K20" s="32" t="n"/>
+      <c r="L20" s="32" t="n"/>
+      <c r="M20" s="32" t="n"/>
+      <c r="N20" s="33" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="43" t="n"/>
-      <c r="B21" s="30" t="n"/>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="A21" s="41" t="n"/>
+      <c r="B21" s="28" t="n"/>
+      <c r="C21" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D21" s="32" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="34" t="n"/>
-      <c r="G21" s="34" t="n"/>
-      <c r="H21" s="34" t="n"/>
-      <c r="I21" s="34" t="n"/>
-      <c r="J21" s="34" t="n"/>
-      <c r="K21" s="34" t="n"/>
-      <c r="L21" s="34" t="n"/>
-      <c r="M21" s="34" t="n"/>
-      <c r="N21" s="35" t="n"/>
+      <c r="D21" s="30" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n"/>
+      <c r="K21" s="32" t="n"/>
+      <c r="L21" s="32" t="n"/>
+      <c r="M21" s="32" t="n"/>
+      <c r="N21" s="33" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="44" t="n"/>
-      <c r="B22" s="37" t="inlineStr">
+      <c r="A22" s="42" t="n"/>
+      <c r="B22" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C22" s="38" t="inlineStr">
+      <c r="C22" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D22" s="39" t="n"/>
-      <c r="E22" s="40" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="41" t="n"/>
-      <c r="I22" s="41" t="n"/>
-      <c r="J22" s="41" t="n"/>
-      <c r="K22" s="41" t="n"/>
-      <c r="L22" s="41" t="n"/>
-      <c r="M22" s="41" t="n"/>
-      <c r="N22" s="42" t="n"/>
+      <c r="D22" s="37" t="n"/>
+      <c r="E22" s="38" t="n"/>
+      <c r="F22" s="39" t="n"/>
+      <c r="G22" s="39" t="n"/>
+      <c r="H22" s="39" t="n"/>
+      <c r="I22" s="39" t="n"/>
+      <c r="J22" s="39" t="n"/>
+      <c r="K22" s="39" t="n"/>
+      <c r="L22" s="39" t="n"/>
+      <c r="M22" s="39" t="n"/>
+      <c r="N22" s="40" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="29" t="n"/>
-      <c r="B23" s="30" t="n"/>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="A23" s="27" t="n"/>
+      <c r="B23" s="28" t="n"/>
+      <c r="C23" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D23" s="32" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="34" t="n"/>
-      <c r="G23" s="34" t="n"/>
-      <c r="H23" s="34" t="n"/>
-      <c r="I23" s="34" t="n"/>
-      <c r="J23" s="34" t="n"/>
-      <c r="K23" s="34" t="n"/>
-      <c r="L23" s="34" t="n"/>
-      <c r="M23" s="34" t="n"/>
-      <c r="N23" s="35" t="n"/>
+      <c r="D23" s="30" t="n"/>
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="32" t="n"/>
+      <c r="I23" s="32" t="n"/>
+      <c r="J23" s="32" t="n"/>
+      <c r="K23" s="32" t="n"/>
+      <c r="L23" s="32" t="n"/>
+      <c r="M23" s="32" t="n"/>
+      <c r="N23" s="33" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="n"/>
-      <c r="C24" s="47" t="inlineStr">
+      <c r="A24" s="43" t="n"/>
+      <c r="B24" s="44" t="n"/>
+      <c r="C24" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D24" s="48" t="n"/>
-      <c r="E24" s="49" t="n"/>
-      <c r="F24" s="50" t="n"/>
-      <c r="G24" s="50" t="n"/>
-      <c r="H24" s="50" t="n"/>
-      <c r="I24" s="50" t="n"/>
-      <c r="J24" s="50" t="n"/>
-      <c r="K24" s="50" t="n"/>
-      <c r="L24" s="50" t="n"/>
-      <c r="M24" s="50" t="n"/>
-      <c r="N24" s="51" t="n"/>
+      <c r="D24" s="46" t="n"/>
+      <c r="E24" s="47" t="n"/>
+      <c r="F24" s="48" t="n"/>
+      <c r="G24" s="48" t="n"/>
+      <c r="H24" s="48" t="n"/>
+      <c r="I24" s="48" t="n"/>
+      <c r="J24" s="48" t="n"/>
+      <c r="K24" s="48" t="n"/>
+      <c r="L24" s="48" t="n"/>
+      <c r="M24" s="48" t="n"/>
+      <c r="N24" s="49" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="22" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D25" s="25" t="n"/>
-      <c r="E25" s="26" t="n"/>
-      <c r="F25" s="27" t="n"/>
-      <c r="G25" s="27" t="n"/>
-      <c r="H25" s="27" t="n"/>
-      <c r="I25" s="27" t="n"/>
-      <c r="J25" s="27" t="n"/>
-      <c r="K25" s="27" t="n"/>
-      <c r="L25" s="27" t="n"/>
-      <c r="M25" s="27" t="n"/>
-      <c r="N25" s="28" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+      <c r="K25" s="25" t="n"/>
+      <c r="L25" s="25" t="n"/>
+      <c r="M25" s="25" t="n"/>
+      <c r="N25" s="26" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="29" t="n"/>
-      <c r="B26" s="30" t="n"/>
-      <c r="C26" s="31" t="inlineStr">
+      <c r="A26" s="27" t="n"/>
+      <c r="B26" s="28" t="n"/>
+      <c r="C26" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="33" t="n"/>
-      <c r="F26" s="34" t="n"/>
-      <c r="G26" s="34" t="n"/>
-      <c r="H26" s="34" t="n"/>
-      <c r="I26" s="34" t="n"/>
-      <c r="J26" s="34" t="n"/>
-      <c r="K26" s="34" t="n"/>
-      <c r="L26" s="34" t="n"/>
-      <c r="M26" s="34" t="n"/>
-      <c r="N26" s="35" t="n"/>
+      <c r="D26" s="30" t="n"/>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="32" t="n"/>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="32" t="n"/>
+      <c r="J26" s="32" t="n"/>
+      <c r="K26" s="32" t="n"/>
+      <c r="L26" s="32" t="n"/>
+      <c r="M26" s="32" t="n"/>
+      <c r="N26" s="33" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="36" t="n"/>
-      <c r="B27" s="37" t="inlineStr">
+      <c r="A27" s="34" t="n"/>
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C27" s="38" t="inlineStr">
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D27" s="39" t="n"/>
-      <c r="E27" s="40" t="n"/>
-      <c r="F27" s="41" t="n"/>
-      <c r="G27" s="41" t="n"/>
-      <c r="H27" s="41" t="n"/>
-      <c r="I27" s="41" t="n"/>
-      <c r="J27" s="41" t="n"/>
-      <c r="K27" s="41" t="n"/>
-      <c r="L27" s="41" t="n"/>
-      <c r="M27" s="41" t="n"/>
-      <c r="N27" s="42" t="n"/>
+      <c r="D27" s="37" t="n"/>
+      <c r="E27" s="38" t="n"/>
+      <c r="F27" s="39" t="n"/>
+      <c r="G27" s="39" t="n"/>
+      <c r="H27" s="39" t="n"/>
+      <c r="I27" s="39" t="n"/>
+      <c r="J27" s="39" t="n"/>
+      <c r="K27" s="39" t="n"/>
+      <c r="L27" s="39" t="n"/>
+      <c r="M27" s="39" t="n"/>
+      <c r="N27" s="40" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="29" t="n"/>
-      <c r="B28" s="30" t="n"/>
-      <c r="C28" s="31" t="inlineStr">
+      <c r="A28" s="27" t="n"/>
+      <c r="B28" s="28" t="n"/>
+      <c r="C28" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="33" t="n"/>
-      <c r="F28" s="34" t="n"/>
-      <c r="G28" s="34" t="n"/>
-      <c r="H28" s="34" t="n"/>
-      <c r="I28" s="34" t="n"/>
-      <c r="J28" s="34" t="n"/>
-      <c r="K28" s="34" t="n"/>
-      <c r="L28" s="34" t="n"/>
-      <c r="M28" s="34" t="n"/>
-      <c r="N28" s="35" t="n"/>
+      <c r="D28" s="30" t="n"/>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="32" t="n"/>
+      <c r="G28" s="32" t="n"/>
+      <c r="H28" s="32" t="n"/>
+      <c r="I28" s="32" t="n"/>
+      <c r="J28" s="32" t="n"/>
+      <c r="K28" s="32" t="n"/>
+      <c r="L28" s="32" t="n"/>
+      <c r="M28" s="32" t="n"/>
+      <c r="N28" s="33" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="43" t="n"/>
-      <c r="B29" s="30" t="n"/>
-      <c r="C29" s="31" t="inlineStr">
+      <c r="A29" s="41" t="n"/>
+      <c r="B29" s="28" t="n"/>
+      <c r="C29" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="34" t="n"/>
-      <c r="G29" s="34" t="n"/>
-      <c r="H29" s="34" t="n"/>
-      <c r="I29" s="34" t="n"/>
-      <c r="J29" s="34" t="n"/>
-      <c r="K29" s="34" t="n"/>
-      <c r="L29" s="34" t="n"/>
-      <c r="M29" s="34" t="n"/>
-      <c r="N29" s="35" t="n"/>
+      <c r="D29" s="30" t="n"/>
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="32" t="n"/>
+      <c r="G29" s="32" t="n"/>
+      <c r="H29" s="32" t="n"/>
+      <c r="I29" s="32" t="n"/>
+      <c r="J29" s="32" t="n"/>
+      <c r="K29" s="32" t="n"/>
+      <c r="L29" s="32" t="n"/>
+      <c r="M29" s="32" t="n"/>
+      <c r="N29" s="33" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="44" t="n"/>
-      <c r="B30" s="37" t="inlineStr">
+      <c r="A30" s="42" t="n"/>
+      <c r="B30" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C30" s="38" t="inlineStr">
+      <c r="C30" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D30" s="39" t="n"/>
-      <c r="E30" s="40" t="n"/>
-      <c r="F30" s="41" t="n"/>
-      <c r="G30" s="41" t="n"/>
-      <c r="H30" s="41" t="n"/>
-      <c r="I30" s="41" t="n"/>
-      <c r="J30" s="41" t="n"/>
-      <c r="K30" s="41" t="n"/>
-      <c r="L30" s="41" t="n"/>
-      <c r="M30" s="41" t="n"/>
-      <c r="N30" s="42" t="n"/>
+      <c r="D30" s="37" t="n"/>
+      <c r="E30" s="38" t="n"/>
+      <c r="F30" s="39" t="n"/>
+      <c r="G30" s="39" t="n"/>
+      <c r="H30" s="39" t="n"/>
+      <c r="I30" s="39" t="n"/>
+      <c r="J30" s="39" t="n"/>
+      <c r="K30" s="39" t="n"/>
+      <c r="L30" s="39" t="n"/>
+      <c r="M30" s="39" t="n"/>
+      <c r="N30" s="40" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="29" t="n"/>
-      <c r="B31" s="30" t="n"/>
-      <c r="C31" s="31" t="inlineStr">
+      <c r="A31" s="27" t="n"/>
+      <c r="B31" s="28" t="n"/>
+      <c r="C31" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="33" t="n"/>
-      <c r="F31" s="34" t="n"/>
-      <c r="G31" s="34" t="n"/>
-      <c r="H31" s="34" t="n"/>
-      <c r="I31" s="34" t="n"/>
-      <c r="J31" s="34" t="n"/>
-      <c r="K31" s="34" t="n"/>
-      <c r="L31" s="34" t="n"/>
-      <c r="M31" s="34" t="n"/>
-      <c r="N31" s="35" t="n"/>
+      <c r="D31" s="30" t="n"/>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="32" t="n"/>
+      <c r="G31" s="32" t="n"/>
+      <c r="H31" s="32" t="n"/>
+      <c r="I31" s="32" t="n"/>
+      <c r="J31" s="32" t="n"/>
+      <c r="K31" s="32" t="n"/>
+      <c r="L31" s="32" t="n"/>
+      <c r="M31" s="32" t="n"/>
+      <c r="N31" s="33" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="46" t="n"/>
-      <c r="C32" s="47" t="inlineStr">
+      <c r="A32" s="43" t="n"/>
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D32" s="48" t="n"/>
-      <c r="E32" s="49" t="n"/>
-      <c r="F32" s="50" t="n"/>
-      <c r="G32" s="50" t="n"/>
-      <c r="H32" s="50" t="n"/>
-      <c r="I32" s="50" t="n"/>
-      <c r="J32" s="50" t="n"/>
-      <c r="K32" s="50" t="n"/>
-      <c r="L32" s="50" t="n"/>
-      <c r="M32" s="50" t="n"/>
-      <c r="N32" s="51" t="n"/>
+      <c r="D32" s="46" t="n"/>
+      <c r="E32" s="47" t="n"/>
+      <c r="F32" s="48" t="n"/>
+      <c r="G32" s="48" t="n"/>
+      <c r="H32" s="48" t="n"/>
+      <c r="I32" s="48" t="n"/>
+      <c r="J32" s="48" t="n"/>
+      <c r="K32" s="48" t="n"/>
+      <c r="L32" s="48" t="n"/>
+      <c r="M32" s="48" t="n"/>
+      <c r="N32" s="49" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="22" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B33" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C33" s="24" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="26" t="n"/>
-      <c r="F33" s="27" t="n"/>
-      <c r="G33" s="27" t="n"/>
-      <c r="H33" s="27" t="n"/>
-      <c r="I33" s="27" t="n"/>
-      <c r="J33" s="27" t="n"/>
-      <c r="K33" s="27" t="n"/>
-      <c r="L33" s="27" t="n"/>
-      <c r="M33" s="27" t="n"/>
-      <c r="N33" s="28" t="n"/>
+      <c r="D33" s="23" t="n"/>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="25" t="n"/>
+      <c r="G33" s="25" t="n"/>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="25" t="n"/>
+      <c r="J33" s="25" t="n"/>
+      <c r="K33" s="25" t="n"/>
+      <c r="L33" s="25" t="n"/>
+      <c r="M33" s="25" t="n"/>
+      <c r="N33" s="26" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="29" t="n"/>
-      <c r="B34" s="30" t="n"/>
-      <c r="C34" s="31" t="inlineStr">
+      <c r="A34" s="27" t="n"/>
+      <c r="B34" s="28" t="n"/>
+      <c r="C34" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D34" s="32" t="n"/>
-      <c r="E34" s="33" t="n"/>
-      <c r="F34" s="34" t="n"/>
-      <c r="G34" s="34" t="n"/>
-      <c r="H34" s="34" t="n"/>
-      <c r="I34" s="34" t="n"/>
-      <c r="J34" s="34" t="n"/>
-      <c r="K34" s="34" t="n"/>
-      <c r="L34" s="34" t="n"/>
-      <c r="M34" s="34" t="n"/>
-      <c r="N34" s="35" t="n"/>
+      <c r="D34" s="30" t="n"/>
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="32" t="n"/>
+      <c r="G34" s="32" t="n"/>
+      <c r="H34" s="32" t="n"/>
+      <c r="I34" s="32" t="n"/>
+      <c r="J34" s="32" t="n"/>
+      <c r="K34" s="32" t="n"/>
+      <c r="L34" s="32" t="n"/>
+      <c r="M34" s="32" t="n"/>
+      <c r="N34" s="33" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="36" t="n"/>
-      <c r="B35" s="37" t="inlineStr">
+      <c r="A35" s="34" t="n"/>
+      <c r="B35" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C35" s="38" t="inlineStr">
+      <c r="C35" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D35" s="39" t="n"/>
-      <c r="E35" s="40" t="n"/>
-      <c r="F35" s="41" t="n"/>
-      <c r="G35" s="41" t="n"/>
-      <c r="H35" s="41" t="n"/>
-      <c r="I35" s="41" t="n"/>
-      <c r="J35" s="41" t="n"/>
-      <c r="K35" s="41" t="n"/>
-      <c r="L35" s="41" t="n"/>
-      <c r="M35" s="41" t="n"/>
-      <c r="N35" s="42" t="n"/>
+      <c r="D35" s="37" t="n"/>
+      <c r="E35" s="38" t="n"/>
+      <c r="F35" s="39" t="n"/>
+      <c r="G35" s="39" t="n"/>
+      <c r="H35" s="39" t="n"/>
+      <c r="I35" s="39" t="n"/>
+      <c r="J35" s="39" t="n"/>
+      <c r="K35" s="39" t="n"/>
+      <c r="L35" s="39" t="n"/>
+      <c r="M35" s="39" t="n"/>
+      <c r="N35" s="40" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="29" t="n"/>
-      <c r="B36" s="30" t="n"/>
-      <c r="C36" s="31" t="inlineStr">
+      <c r="A36" s="27" t="n"/>
+      <c r="B36" s="28" t="n"/>
+      <c r="C36" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D36" s="32" t="n"/>
-      <c r="E36" s="33" t="n"/>
-      <c r="F36" s="34" t="n"/>
-      <c r="G36" s="34" t="n"/>
-      <c r="H36" s="34" t="n"/>
-      <c r="I36" s="34" t="n"/>
-      <c r="J36" s="34" t="n"/>
-      <c r="K36" s="34" t="n"/>
-      <c r="L36" s="34" t="n"/>
-      <c r="M36" s="34" t="n"/>
-      <c r="N36" s="35" t="n"/>
+      <c r="D36" s="30" t="n"/>
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="32" t="n"/>
+      <c r="G36" s="32" t="n"/>
+      <c r="H36" s="32" t="n"/>
+      <c r="I36" s="32" t="n"/>
+      <c r="J36" s="32" t="n"/>
+      <c r="K36" s="32" t="n"/>
+      <c r="L36" s="32" t="n"/>
+      <c r="M36" s="32" t="n"/>
+      <c r="N36" s="33" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="43" t="n"/>
-      <c r="B37" s="30" t="n"/>
-      <c r="C37" s="31" t="inlineStr">
+      <c r="A37" s="41" t="n"/>
+      <c r="B37" s="28" t="n"/>
+      <c r="C37" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D37" s="32" t="n"/>
-      <c r="E37" s="33" t="n"/>
-      <c r="F37" s="34" t="n"/>
-      <c r="G37" s="34" t="n"/>
-      <c r="H37" s="34" t="n"/>
-      <c r="I37" s="34" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="34" t="n"/>
-      <c r="L37" s="34" t="n"/>
-      <c r="M37" s="34" t="n"/>
-      <c r="N37" s="35" t="n"/>
+      <c r="D37" s="30" t="n"/>
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="32" t="n"/>
+      <c r="J37" s="32" t="n"/>
+      <c r="K37" s="32" t="n"/>
+      <c r="L37" s="32" t="n"/>
+      <c r="M37" s="32" t="n"/>
+      <c r="N37" s="33" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="44" t="n"/>
-      <c r="B38" s="37" t="inlineStr">
+      <c r="A38" s="42" t="n"/>
+      <c r="B38" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C38" s="38" t="inlineStr">
+      <c r="C38" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D38" s="39" t="n"/>
-      <c r="E38" s="40" t="n"/>
-      <c r="F38" s="41" t="n"/>
-      <c r="G38" s="41" t="n"/>
-      <c r="H38" s="41" t="n"/>
-      <c r="I38" s="41" t="n"/>
-      <c r="J38" s="41" t="n"/>
-      <c r="K38" s="41" t="n"/>
-      <c r="L38" s="41" t="n"/>
-      <c r="M38" s="41" t="n"/>
-      <c r="N38" s="42" t="n"/>
+      <c r="D38" s="37" t="n"/>
+      <c r="E38" s="38" t="n"/>
+      <c r="F38" s="39" t="n"/>
+      <c r="G38" s="39" t="n"/>
+      <c r="H38" s="39" t="n"/>
+      <c r="I38" s="39" t="n"/>
+      <c r="J38" s="39" t="n"/>
+      <c r="K38" s="39" t="n"/>
+      <c r="L38" s="39" t="n"/>
+      <c r="M38" s="39" t="n"/>
+      <c r="N38" s="40" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="29" t="n"/>
-      <c r="B39" s="30" t="n"/>
-      <c r="C39" s="31" t="inlineStr">
+      <c r="A39" s="27" t="n"/>
+      <c r="B39" s="28" t="n"/>
+      <c r="C39" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D39" s="32" t="n"/>
-      <c r="E39" s="33" t="n"/>
-      <c r="F39" s="34" t="n"/>
-      <c r="G39" s="34" t="n"/>
-      <c r="H39" s="34" t="n"/>
-      <c r="I39" s="34" t="n"/>
-      <c r="J39" s="34" t="n"/>
-      <c r="K39" s="34" t="n"/>
-      <c r="L39" s="34" t="n"/>
-      <c r="M39" s="34" t="n"/>
-      <c r="N39" s="35" t="n"/>
+      <c r="D39" s="30" t="n"/>
+      <c r="E39" s="31" t="n"/>
+      <c r="F39" s="32" t="n"/>
+      <c r="G39" s="32" t="n"/>
+      <c r="H39" s="32" t="n"/>
+      <c r="I39" s="32" t="n"/>
+      <c r="J39" s="32" t="n"/>
+      <c r="K39" s="32" t="n"/>
+      <c r="L39" s="32" t="n"/>
+      <c r="M39" s="32" t="n"/>
+      <c r="N39" s="33" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="n"/>
-      <c r="C40" s="47" t="inlineStr">
+      <c r="A40" s="43" t="n"/>
+      <c r="B40" s="44" t="n"/>
+      <c r="C40" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D40" s="48" t="n"/>
-      <c r="E40" s="49" t="n"/>
-      <c r="F40" s="50" t="n"/>
-      <c r="G40" s="50" t="n"/>
-      <c r="H40" s="50" t="n"/>
-      <c r="I40" s="50" t="n"/>
-      <c r="J40" s="50" t="n"/>
-      <c r="K40" s="50" t="n"/>
-      <c r="L40" s="50" t="n"/>
-      <c r="M40" s="50" t="n"/>
-      <c r="N40" s="51" t="n"/>
+      <c r="D40" s="46" t="n"/>
+      <c r="E40" s="47" t="n"/>
+      <c r="F40" s="48" t="n"/>
+      <c r="G40" s="48" t="n"/>
+      <c r="H40" s="48" t="n"/>
+      <c r="I40" s="48" t="n"/>
+      <c r="J40" s="48" t="n"/>
+      <c r="K40" s="48" t="n"/>
+      <c r="L40" s="48" t="n"/>
+      <c r="M40" s="48" t="n"/>
+      <c r="N40" s="49" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="22" t="inlineStr">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B41" s="23" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C41" s="24" t="inlineStr">
+      <c r="C41" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D41" s="25" t="n"/>
-      <c r="E41" s="26" t="n"/>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
-      <c r="H41" s="27" t="n"/>
-      <c r="I41" s="27" t="n"/>
-      <c r="J41" s="27" t="n"/>
-      <c r="K41" s="27" t="n"/>
-      <c r="L41" s="27" t="n"/>
-      <c r="M41" s="27" t="n"/>
-      <c r="N41" s="28" t="n"/>
+      <c r="D41" s="23" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
+      <c r="J41" s="25" t="n"/>
+      <c r="K41" s="25" t="n"/>
+      <c r="L41" s="25" t="n"/>
+      <c r="M41" s="25" t="n"/>
+      <c r="N41" s="26" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="29" t="n"/>
-      <c r="B42" s="30" t="n"/>
-      <c r="C42" s="31" t="inlineStr">
+      <c r="A42" s="27" t="n"/>
+      <c r="B42" s="28" t="n"/>
+      <c r="C42" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D42" s="32" t="n"/>
-      <c r="E42" s="33" t="n"/>
-      <c r="F42" s="34" t="n"/>
-      <c r="G42" s="34" t="n"/>
-      <c r="H42" s="34" t="n"/>
-      <c r="I42" s="34" t="n"/>
-      <c r="J42" s="34" t="n"/>
-      <c r="K42" s="34" t="n"/>
-      <c r="L42" s="34" t="n"/>
-      <c r="M42" s="34" t="n"/>
-      <c r="N42" s="35" t="n"/>
+      <c r="D42" s="30" t="n"/>
+      <c r="E42" s="31" t="n"/>
+      <c r="F42" s="32" t="n"/>
+      <c r="G42" s="32" t="n"/>
+      <c r="H42" s="32" t="n"/>
+      <c r="I42" s="32" t="n"/>
+      <c r="J42" s="32" t="n"/>
+      <c r="K42" s="32" t="n"/>
+      <c r="L42" s="32" t="n"/>
+      <c r="M42" s="32" t="n"/>
+      <c r="N42" s="33" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="36" t="n"/>
-      <c r="B43" s="37" t="inlineStr">
+      <c r="A43" s="34" t="n"/>
+      <c r="B43" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C43" s="38" t="inlineStr">
+      <c r="C43" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D43" s="39" t="n"/>
-      <c r="E43" s="40" t="n"/>
-      <c r="F43" s="41" t="n"/>
-      <c r="G43" s="41" t="n"/>
-      <c r="H43" s="41" t="n"/>
-      <c r="I43" s="41" t="n"/>
-      <c r="J43" s="41" t="n"/>
-      <c r="K43" s="41" t="n"/>
-      <c r="L43" s="41" t="n"/>
-      <c r="M43" s="41" t="n"/>
-      <c r="N43" s="42" t="n"/>
+      <c r="D43" s="37" t="n"/>
+      <c r="E43" s="38" t="n"/>
+      <c r="F43" s="39" t="n"/>
+      <c r="G43" s="39" t="n"/>
+      <c r="H43" s="39" t="n"/>
+      <c r="I43" s="39" t="n"/>
+      <c r="J43" s="39" t="n"/>
+      <c r="K43" s="39" t="n"/>
+      <c r="L43" s="39" t="n"/>
+      <c r="M43" s="39" t="n"/>
+      <c r="N43" s="40" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="29" t="n"/>
-      <c r="B44" s="30" t="n"/>
-      <c r="C44" s="31" t="inlineStr">
+      <c r="A44" s="27" t="n"/>
+      <c r="B44" s="28" t="n"/>
+      <c r="C44" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D44" s="32" t="n"/>
-      <c r="E44" s="33" t="n"/>
-      <c r="F44" s="34" t="n"/>
-      <c r="G44" s="34" t="n"/>
-      <c r="H44" s="34" t="n"/>
-      <c r="I44" s="34" t="n"/>
-      <c r="J44" s="34" t="n"/>
-      <c r="K44" s="34" t="n"/>
-      <c r="L44" s="34" t="n"/>
-      <c r="M44" s="34" t="n"/>
-      <c r="N44" s="35" t="n"/>
+      <c r="D44" s="30" t="n"/>
+      <c r="E44" s="31" t="n"/>
+      <c r="F44" s="32" t="n"/>
+      <c r="G44" s="32" t="n"/>
+      <c r="H44" s="32" t="n"/>
+      <c r="I44" s="32" t="n"/>
+      <c r="J44" s="32" t="n"/>
+      <c r="K44" s="32" t="n"/>
+      <c r="L44" s="32" t="n"/>
+      <c r="M44" s="32" t="n"/>
+      <c r="N44" s="33" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="43" t="n"/>
-      <c r="B45" s="30" t="n"/>
-      <c r="C45" s="31" t="inlineStr">
+      <c r="A45" s="41" t="n"/>
+      <c r="B45" s="28" t="n"/>
+      <c r="C45" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D45" s="32" t="n"/>
-      <c r="E45" s="33" t="n"/>
-      <c r="F45" s="34" t="n"/>
-      <c r="G45" s="34" t="n"/>
-      <c r="H45" s="34" t="n"/>
-      <c r="I45" s="34" t="n"/>
-      <c r="J45" s="34" t="n"/>
-      <c r="K45" s="34" t="n"/>
-      <c r="L45" s="34" t="n"/>
-      <c r="M45" s="34" t="n"/>
-      <c r="N45" s="35" t="n"/>
+      <c r="D45" s="30" t="n"/>
+      <c r="E45" s="31" t="n"/>
+      <c r="F45" s="32" t="n"/>
+      <c r="G45" s="32" t="n"/>
+      <c r="H45" s="32" t="n"/>
+      <c r="I45" s="32" t="n"/>
+      <c r="J45" s="32" t="n"/>
+      <c r="K45" s="32" t="n"/>
+      <c r="L45" s="32" t="n"/>
+      <c r="M45" s="32" t="n"/>
+      <c r="N45" s="33" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="44" t="n"/>
-      <c r="B46" s="37" t="inlineStr">
+      <c r="A46" s="42" t="n"/>
+      <c r="B46" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C46" s="38" t="inlineStr">
+      <c r="C46" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D46" s="39" t="n"/>
-      <c r="E46" s="40" t="n"/>
-      <c r="F46" s="41" t="n"/>
-      <c r="G46" s="41" t="n"/>
-      <c r="H46" s="41" t="n"/>
-      <c r="I46" s="41" t="n"/>
-      <c r="J46" s="41" t="n"/>
-      <c r="K46" s="41" t="n"/>
-      <c r="L46" s="41" t="n"/>
-      <c r="M46" s="41" t="n"/>
-      <c r="N46" s="42" t="n"/>
+      <c r="D46" s="37" t="n"/>
+      <c r="E46" s="38" t="n"/>
+      <c r="F46" s="39" t="n"/>
+      <c r="G46" s="39" t="n"/>
+      <c r="H46" s="39" t="n"/>
+      <c r="I46" s="39" t="n"/>
+      <c r="J46" s="39" t="n"/>
+      <c r="K46" s="39" t="n"/>
+      <c r="L46" s="39" t="n"/>
+      <c r="M46" s="39" t="n"/>
+      <c r="N46" s="40" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="29" t="n"/>
-      <c r="B47" s="30" t="n"/>
-      <c r="C47" s="31" t="inlineStr">
+      <c r="A47" s="27" t="n"/>
+      <c r="B47" s="28" t="n"/>
+      <c r="C47" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D47" s="32" t="n"/>
-      <c r="E47" s="33" t="n"/>
-      <c r="F47" s="34" t="n"/>
-      <c r="G47" s="34" t="n"/>
-      <c r="H47" s="34" t="n"/>
-      <c r="I47" s="34" t="n"/>
-      <c r="J47" s="34" t="n"/>
-      <c r="K47" s="34" t="n"/>
-      <c r="L47" s="34" t="n"/>
-      <c r="M47" s="34" t="n"/>
-      <c r="N47" s="35" t="n"/>
+      <c r="D47" s="30" t="n"/>
+      <c r="E47" s="31" t="n"/>
+      <c r="F47" s="32" t="n"/>
+      <c r="G47" s="32" t="n"/>
+      <c r="H47" s="32" t="n"/>
+      <c r="I47" s="32" t="n"/>
+      <c r="J47" s="32" t="n"/>
+      <c r="K47" s="32" t="n"/>
+      <c r="L47" s="32" t="n"/>
+      <c r="M47" s="32" t="n"/>
+      <c r="N47" s="33" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="45" t="n"/>
-      <c r="B48" s="46" t="n"/>
-      <c r="C48" s="47" t="inlineStr">
+      <c r="A48" s="43" t="n"/>
+      <c r="B48" s="44" t="n"/>
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D48" s="48" t="n"/>
-      <c r="E48" s="49" t="n"/>
-      <c r="F48" s="50" t="n"/>
-      <c r="G48" s="50" t="n"/>
-      <c r="H48" s="50" t="n"/>
-      <c r="I48" s="50" t="n"/>
-      <c r="J48" s="50" t="n"/>
-      <c r="K48" s="50" t="n"/>
-      <c r="L48" s="50" t="n"/>
-      <c r="M48" s="50" t="n"/>
-      <c r="N48" s="51" t="n"/>
+      <c r="D48" s="46" t="n"/>
+      <c r="E48" s="47" t="n"/>
+      <c r="F48" s="48" t="n"/>
+      <c r="G48" s="48" t="n"/>
+      <c r="H48" s="48" t="n"/>
+      <c r="I48" s="48" t="n"/>
+      <c r="J48" s="48" t="n"/>
+      <c r="K48" s="48" t="n"/>
+      <c r="L48" s="48" t="n"/>
+      <c r="M48" s="48" t="n"/>
+      <c r="N48" s="49" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="22" t="inlineStr">
+      <c r="A49" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B49" s="23" t="inlineStr">
+      <c r="B49" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C49" s="24" t="inlineStr">
+      <c r="C49" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D49" s="25" t="n"/>
-      <c r="E49" s="26" t="n"/>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="27" t="n"/>
-      <c r="I49" s="27" t="n"/>
-      <c r="J49" s="27" t="n"/>
-      <c r="K49" s="27" t="n"/>
-      <c r="L49" s="27" t="n"/>
-      <c r="M49" s="27" t="n"/>
-      <c r="N49" s="28" t="n"/>
+      <c r="D49" s="23" t="n"/>
+      <c r="E49" s="24" t="n"/>
+      <c r="F49" s="25" t="n"/>
+      <c r="G49" s="25" t="n"/>
+      <c r="H49" s="25" t="n"/>
+      <c r="I49" s="25" t="n"/>
+      <c r="J49" s="25" t="n"/>
+      <c r="K49" s="25" t="n"/>
+      <c r="L49" s="25" t="n"/>
+      <c r="M49" s="25" t="n"/>
+      <c r="N49" s="26" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="29" t="n"/>
-      <c r="B50" s="30" t="n"/>
-      <c r="C50" s="31" t="inlineStr">
+      <c r="A50" s="27" t="n"/>
+      <c r="B50" s="28" t="n"/>
+      <c r="C50" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D50" s="32" t="n"/>
-      <c r="E50" s="33" t="n"/>
-      <c r="F50" s="34" t="n"/>
-      <c r="G50" s="34" t="n"/>
-      <c r="H50" s="34" t="n"/>
-      <c r="I50" s="34" t="n"/>
-      <c r="J50" s="34" t="n"/>
-      <c r="K50" s="34" t="n"/>
-      <c r="L50" s="34" t="n"/>
-      <c r="M50" s="34" t="n"/>
-      <c r="N50" s="35" t="n"/>
+      <c r="D50" s="30" t="n"/>
+      <c r="E50" s="31" t="n"/>
+      <c r="F50" s="32" t="n"/>
+      <c r="G50" s="32" t="n"/>
+      <c r="H50" s="32" t="n"/>
+      <c r="I50" s="32" t="n"/>
+      <c r="J50" s="32" t="n"/>
+      <c r="K50" s="32" t="n"/>
+      <c r="L50" s="32" t="n"/>
+      <c r="M50" s="32" t="n"/>
+      <c r="N50" s="33" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="36" t="n"/>
-      <c r="B51" s="37" t="inlineStr">
+      <c r="A51" s="34" t="n"/>
+      <c r="B51" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C51" s="38" t="inlineStr">
+      <c r="C51" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D51" s="39" t="n"/>
-      <c r="E51" s="40" t="n"/>
-      <c r="F51" s="41" t="n"/>
-      <c r="G51" s="41" t="n"/>
-      <c r="H51" s="41" t="n"/>
-      <c r="I51" s="41" t="n"/>
-      <c r="J51" s="41" t="n"/>
-      <c r="K51" s="41" t="n"/>
-      <c r="L51" s="41" t="n"/>
-      <c r="M51" s="41" t="n"/>
-      <c r="N51" s="42" t="n"/>
+      <c r="D51" s="37" t="n"/>
+      <c r="E51" s="38" t="n"/>
+      <c r="F51" s="39" t="n"/>
+      <c r="G51" s="39" t="n"/>
+      <c r="H51" s="39" t="n"/>
+      <c r="I51" s="39" t="n"/>
+      <c r="J51" s="39" t="n"/>
+      <c r="K51" s="39" t="n"/>
+      <c r="L51" s="39" t="n"/>
+      <c r="M51" s="39" t="n"/>
+      <c r="N51" s="40" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="29" t="n"/>
-      <c r="B52" s="30" t="n"/>
-      <c r="C52" s="31" t="inlineStr">
+      <c r="A52" s="27" t="n"/>
+      <c r="B52" s="28" t="n"/>
+      <c r="C52" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D52" s="32" t="n"/>
-      <c r="E52" s="33" t="n"/>
-      <c r="F52" s="34" t="n"/>
-      <c r="G52" s="34" t="n"/>
-      <c r="H52" s="34" t="n"/>
-      <c r="I52" s="34" t="n"/>
-      <c r="J52" s="34" t="n"/>
-      <c r="K52" s="34" t="n"/>
-      <c r="L52" s="34" t="n"/>
-      <c r="M52" s="34" t="n"/>
-      <c r="N52" s="35" t="n"/>
+      <c r="D52" s="30" t="n"/>
+      <c r="E52" s="31" t="n"/>
+      <c r="F52" s="32" t="n"/>
+      <c r="G52" s="32" t="n"/>
+      <c r="H52" s="32" t="n"/>
+      <c r="I52" s="32" t="n"/>
+      <c r="J52" s="32" t="n"/>
+      <c r="K52" s="32" t="n"/>
+      <c r="L52" s="32" t="n"/>
+      <c r="M52" s="32" t="n"/>
+      <c r="N52" s="33" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="43" t="n"/>
-      <c r="B53" s="30" t="n"/>
-      <c r="C53" s="31" t="inlineStr">
+      <c r="A53" s="41" t="n"/>
+      <c r="B53" s="28" t="n"/>
+      <c r="C53" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D53" s="32" t="n"/>
-      <c r="E53" s="33" t="n"/>
-      <c r="F53" s="34" t="n"/>
-      <c r="G53" s="34" t="n"/>
-      <c r="H53" s="34" t="n"/>
-      <c r="I53" s="34" t="n"/>
-      <c r="J53" s="34" t="n"/>
-      <c r="K53" s="34" t="n"/>
-      <c r="L53" s="34" t="n"/>
-      <c r="M53" s="34" t="n"/>
-      <c r="N53" s="35" t="n"/>
+      <c r="D53" s="30" t="n"/>
+      <c r="E53" s="31" t="n"/>
+      <c r="F53" s="32" t="n"/>
+      <c r="G53" s="32" t="n"/>
+      <c r="H53" s="32" t="n"/>
+      <c r="I53" s="32" t="n"/>
+      <c r="J53" s="32" t="n"/>
+      <c r="K53" s="32" t="n"/>
+      <c r="L53" s="32" t="n"/>
+      <c r="M53" s="32" t="n"/>
+      <c r="N53" s="33" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="44" t="n"/>
-      <c r="B54" s="37" t="inlineStr">
+      <c r="A54" s="42" t="n"/>
+      <c r="B54" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C54" s="38" t="inlineStr">
+      <c r="C54" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D54" s="39" t="n"/>
-      <c r="E54" s="40" t="n"/>
-      <c r="F54" s="41" t="n"/>
-      <c r="G54" s="41" t="n"/>
-      <c r="H54" s="41" t="n"/>
-      <c r="I54" s="41" t="n"/>
-      <c r="J54" s="41" t="n"/>
-      <c r="K54" s="41" t="n"/>
-      <c r="L54" s="41" t="n"/>
-      <c r="M54" s="41" t="n"/>
-      <c r="N54" s="42" t="n"/>
+      <c r="D54" s="37" t="n"/>
+      <c r="E54" s="38" t="n"/>
+      <c r="F54" s="39" t="n"/>
+      <c r="G54" s="39" t="n"/>
+      <c r="H54" s="39" t="n"/>
+      <c r="I54" s="39" t="n"/>
+      <c r="J54" s="39" t="n"/>
+      <c r="K54" s="39" t="n"/>
+      <c r="L54" s="39" t="n"/>
+      <c r="M54" s="39" t="n"/>
+      <c r="N54" s="40" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="29" t="n"/>
-      <c r="B55" s="30" t="n"/>
-      <c r="C55" s="31" t="inlineStr">
+      <c r="A55" s="27" t="n"/>
+      <c r="B55" s="28" t="n"/>
+      <c r="C55" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D55" s="32" t="n"/>
-      <c r="E55" s="33" t="n"/>
-      <c r="F55" s="34" t="n"/>
-      <c r="G55" s="34" t="n"/>
-      <c r="H55" s="34" t="n"/>
-      <c r="I55" s="34" t="n"/>
-      <c r="J55" s="34" t="n"/>
-      <c r="K55" s="34" t="n"/>
-      <c r="L55" s="34" t="n"/>
-      <c r="M55" s="34" t="n"/>
-      <c r="N55" s="35" t="n"/>
+      <c r="D55" s="30" t="n"/>
+      <c r="E55" s="31" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="32" t="n"/>
+      <c r="H55" s="32" t="n"/>
+      <c r="I55" s="32" t="n"/>
+      <c r="J55" s="32" t="n"/>
+      <c r="K55" s="32" t="n"/>
+      <c r="L55" s="32" t="n"/>
+      <c r="M55" s="32" t="n"/>
+      <c r="N55" s="33" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="45" t="n"/>
-      <c r="B56" s="46" t="n"/>
-      <c r="C56" s="47" t="inlineStr">
+      <c r="A56" s="43" t="n"/>
+      <c r="B56" s="44" t="n"/>
+      <c r="C56" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D56" s="48" t="n"/>
-      <c r="E56" s="49" t="n"/>
-      <c r="F56" s="50" t="n"/>
-      <c r="G56" s="50" t="n"/>
-      <c r="H56" s="50" t="n"/>
-      <c r="I56" s="50" t="n"/>
-      <c r="J56" s="50" t="n"/>
-      <c r="K56" s="50" t="n"/>
-      <c r="L56" s="50" t="n"/>
-      <c r="M56" s="50" t="n"/>
-      <c r="N56" s="51" t="n"/>
+      <c r="D56" s="46" t="n"/>
+      <c r="E56" s="47" t="n"/>
+      <c r="F56" s="48" t="n"/>
+      <c r="G56" s="48" t="n"/>
+      <c r="H56" s="48" t="n"/>
+      <c r="I56" s="48" t="n"/>
+      <c r="J56" s="48" t="n"/>
+      <c r="K56" s="48" t="n"/>
+      <c r="L56" s="48" t="n"/>
+      <c r="M56" s="48" t="n"/>
+      <c r="N56" s="49" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+      <c r="A57" s="20" t="inlineStr">
         <is>
           <t>（　）</t>
         </is>
       </c>
-      <c r="B57" s="23" t="inlineStr">
+      <c r="B57" s="21" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C57" s="24" t="inlineStr">
+      <c r="C57" s="22" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D57" s="25" t="n"/>
-      <c r="E57" s="26" t="n"/>
-      <c r="F57" s="27" t="n"/>
-      <c r="G57" s="27" t="n"/>
-      <c r="H57" s="27" t="n"/>
-      <c r="I57" s="27" t="n"/>
-      <c r="J57" s="27" t="n"/>
-      <c r="K57" s="27" t="n"/>
-      <c r="L57" s="27" t="n"/>
-      <c r="M57" s="27" t="n"/>
-      <c r="N57" s="28" t="n"/>
+      <c r="D57" s="23" t="n"/>
+      <c r="E57" s="24" t="n"/>
+      <c r="F57" s="25" t="n"/>
+      <c r="G57" s="25" t="n"/>
+      <c r="H57" s="25" t="n"/>
+      <c r="I57" s="25" t="n"/>
+      <c r="J57" s="25" t="n"/>
+      <c r="K57" s="25" t="n"/>
+      <c r="L57" s="25" t="n"/>
+      <c r="M57" s="25" t="n"/>
+      <c r="N57" s="26" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="29" t="n"/>
-      <c r="B58" s="30" t="n"/>
-      <c r="C58" s="31" t="inlineStr">
+      <c r="A58" s="27" t="n"/>
+      <c r="B58" s="28" t="n"/>
+      <c r="C58" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D58" s="32" t="n"/>
-      <c r="E58" s="33" t="n"/>
-      <c r="F58" s="34" t="n"/>
-      <c r="G58" s="34" t="n"/>
-      <c r="H58" s="34" t="n"/>
-      <c r="I58" s="34" t="n"/>
-      <c r="J58" s="34" t="n"/>
-      <c r="K58" s="34" t="n"/>
-      <c r="L58" s="34" t="n"/>
-      <c r="M58" s="34" t="n"/>
-      <c r="N58" s="35" t="n"/>
+      <c r="D58" s="30" t="n"/>
+      <c r="E58" s="31" t="n"/>
+      <c r="F58" s="32" t="n"/>
+      <c r="G58" s="32" t="n"/>
+      <c r="H58" s="32" t="n"/>
+      <c r="I58" s="32" t="n"/>
+      <c r="J58" s="32" t="n"/>
+      <c r="K58" s="32" t="n"/>
+      <c r="L58" s="32" t="n"/>
+      <c r="M58" s="32" t="n"/>
+      <c r="N58" s="33" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="36" t="n"/>
-      <c r="B59" s="37" t="inlineStr">
+      <c r="A59" s="34" t="n"/>
+      <c r="B59" s="35" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="C59" s="38" t="inlineStr">
+      <c r="C59" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D59" s="39" t="n"/>
-      <c r="E59" s="40" t="n"/>
-      <c r="F59" s="41" t="n"/>
-      <c r="G59" s="41" t="n"/>
-      <c r="H59" s="41" t="n"/>
-      <c r="I59" s="41" t="n"/>
-      <c r="J59" s="41" t="n"/>
-      <c r="K59" s="41" t="n"/>
-      <c r="L59" s="41" t="n"/>
-      <c r="M59" s="41" t="n"/>
-      <c r="N59" s="42" t="n"/>
+      <c r="D59" s="37" t="n"/>
+      <c r="E59" s="38" t="n"/>
+      <c r="F59" s="39" t="n"/>
+      <c r="G59" s="39" t="n"/>
+      <c r="H59" s="39" t="n"/>
+      <c r="I59" s="39" t="n"/>
+      <c r="J59" s="39" t="n"/>
+      <c r="K59" s="39" t="n"/>
+      <c r="L59" s="39" t="n"/>
+      <c r="M59" s="39" t="n"/>
+      <c r="N59" s="40" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="29" t="n"/>
-      <c r="B60" s="30" t="n"/>
-      <c r="C60" s="31" t="inlineStr">
+      <c r="A60" s="27" t="n"/>
+      <c r="B60" s="28" t="n"/>
+      <c r="C60" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D60" s="32" t="n"/>
-      <c r="E60" s="33" t="n"/>
-      <c r="F60" s="34" t="n"/>
-      <c r="G60" s="34" t="n"/>
-      <c r="H60" s="34" t="n"/>
-      <c r="I60" s="34" t="n"/>
-      <c r="J60" s="34" t="n"/>
-      <c r="K60" s="34" t="n"/>
-      <c r="L60" s="34" t="n"/>
-      <c r="M60" s="34" t="n"/>
-      <c r="N60" s="35" t="n"/>
+      <c r="D60" s="30" t="n"/>
+      <c r="E60" s="31" t="n"/>
+      <c r="F60" s="32" t="n"/>
+      <c r="G60" s="32" t="n"/>
+      <c r="H60" s="32" t="n"/>
+      <c r="I60" s="32" t="n"/>
+      <c r="J60" s="32" t="n"/>
+      <c r="K60" s="32" t="n"/>
+      <c r="L60" s="32" t="n"/>
+      <c r="M60" s="32" t="n"/>
+      <c r="N60" s="33" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="43" t="n"/>
-      <c r="B61" s="30" t="n"/>
-      <c r="C61" s="31" t="inlineStr">
+      <c r="A61" s="41" t="n"/>
+      <c r="B61" s="28" t="n"/>
+      <c r="C61" s="29" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D61" s="32" t="n"/>
-      <c r="E61" s="33" t="n"/>
-      <c r="F61" s="34" t="n"/>
-      <c r="G61" s="34" t="n"/>
-      <c r="H61" s="34" t="n"/>
-      <c r="I61" s="34" t="n"/>
-      <c r="J61" s="34" t="n"/>
-      <c r="K61" s="34" t="n"/>
-      <c r="L61" s="34" t="n"/>
-      <c r="M61" s="34" t="n"/>
-      <c r="N61" s="35" t="n"/>
+      <c r="D61" s="30" t="n"/>
+      <c r="E61" s="31" t="n"/>
+      <c r="F61" s="32" t="n"/>
+      <c r="G61" s="32" t="n"/>
+      <c r="H61" s="32" t="n"/>
+      <c r="I61" s="32" t="n"/>
+      <c r="J61" s="32" t="n"/>
+      <c r="K61" s="32" t="n"/>
+      <c r="L61" s="32" t="n"/>
+      <c r="M61" s="32" t="n"/>
+      <c r="N61" s="33" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="44" t="n"/>
-      <c r="B62" s="37" t="inlineStr">
+      <c r="A62" s="42" t="n"/>
+      <c r="B62" s="35" t="inlineStr">
         <is>
           <t>夕</t>
         </is>
       </c>
-      <c r="C62" s="38" t="inlineStr">
+      <c r="C62" s="36" t="inlineStr">
         <is>
           <t>主</t>
         </is>
       </c>
-      <c r="D62" s="39" t="n"/>
-      <c r="E62" s="40" t="n"/>
-      <c r="F62" s="41" t="n"/>
-      <c r="G62" s="41" t="n"/>
-      <c r="H62" s="41" t="n"/>
-      <c r="I62" s="41" t="n"/>
-      <c r="J62" s="41" t="n"/>
-      <c r="K62" s="41" t="n"/>
-      <c r="L62" s="41" t="n"/>
-      <c r="M62" s="41" t="n"/>
-      <c r="N62" s="42" t="n"/>
+      <c r="D62" s="37" t="n"/>
+      <c r="E62" s="38" t="n"/>
+      <c r="F62" s="39" t="n"/>
+      <c r="G62" s="39" t="n"/>
+      <c r="H62" s="39" t="n"/>
+      <c r="I62" s="39" t="n"/>
+      <c r="J62" s="39" t="n"/>
+      <c r="K62" s="39" t="n"/>
+      <c r="L62" s="39" t="n"/>
+      <c r="M62" s="39" t="n"/>
+      <c r="N62" s="40" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="29" t="n"/>
-      <c r="B63" s="30" t="n"/>
-      <c r="C63" s="31" t="inlineStr">
+      <c r="A63" s="27" t="n"/>
+      <c r="B63" s="28" t="n"/>
+      <c r="C63" s="29" t="inlineStr">
         <is>
           <t>副①</t>
         </is>
       </c>
-      <c r="D63" s="32" t="n"/>
-      <c r="E63" s="33" t="n"/>
-      <c r="F63" s="34" t="n"/>
-      <c r="G63" s="34" t="n"/>
-      <c r="H63" s="34" t="n"/>
-      <c r="I63" s="34" t="n"/>
-      <c r="J63" s="34" t="n"/>
-      <c r="K63" s="34" t="n"/>
-      <c r="L63" s="34" t="n"/>
-      <c r="M63" s="34" t="n"/>
-      <c r="N63" s="35" t="n"/>
+      <c r="D63" s="30" t="n"/>
+      <c r="E63" s="31" t="n"/>
+      <c r="F63" s="32" t="n"/>
+      <c r="G63" s="32" t="n"/>
+      <c r="H63" s="32" t="n"/>
+      <c r="I63" s="32" t="n"/>
+      <c r="J63" s="32" t="n"/>
+      <c r="K63" s="32" t="n"/>
+      <c r="L63" s="32" t="n"/>
+      <c r="M63" s="32" t="n"/>
+      <c r="N63" s="33" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="45" t="n"/>
-      <c r="B64" s="46" t="n"/>
-      <c r="C64" s="47" t="inlineStr">
+      <c r="A64" s="43" t="n"/>
+      <c r="B64" s="44" t="n"/>
+      <c r="C64" s="45" t="inlineStr">
         <is>
           <t>副②</t>
         </is>
       </c>
-      <c r="D64" s="48" t="n"/>
-      <c r="E64" s="49" t="n"/>
-      <c r="F64" s="50" t="n"/>
-      <c r="G64" s="50" t="n"/>
-      <c r="H64" s="50" t="n"/>
-      <c r="I64" s="50" t="n"/>
-      <c r="J64" s="50" t="n"/>
-      <c r="K64" s="50" t="n"/>
-      <c r="L64" s="50" t="n"/>
-      <c r="M64" s="50" t="n"/>
-      <c r="N64" s="52" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="D64" s="46" t="n"/>
+      <c r="E64" s="47" t="n"/>
+      <c r="F64" s="48" t="n"/>
+      <c r="G64" s="48" t="n"/>
+      <c r="H64" s="48" t="n"/>
+      <c r="I64" s="48" t="n"/>
+      <c r="J64" s="48" t="n"/>
+      <c r="K64" s="48" t="n"/>
+      <c r="L64" s="48" t="n"/>
+      <c r="M64" s="48" t="n"/>
+      <c r="N64" s="49" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="38">

</xml_diff>

<commit_message>
Adjust master template generated column widths
</commit_message>
<xml_diff>
--- a/backend/src/data/order_form_master_templates/master_layout_template.xlsx
+++ b/backend/src/data/order_form_master_templates/master_layout_template.xlsx
@@ -70,7 +70,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="57">
     <border>
       <left/>
       <right/>
@@ -574,11 +574,185 @@
       </top>
       <bottom/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -703,6 +877,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -780,58 +965,49 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>225895</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>298932</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>186502</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>312060</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="図 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>5</col>
+      <colOff>225895</colOff>
+      <row>0</row>
+      <rowOff>298932</rowOff>
+    </from>
+    <to>
+      <col>7</col>
+      <colOff>186502</colOff>
+      <row>2</row>
+      <rowOff>312060</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="図 1"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="5721820" y="298932"/>
           <a:ext cx="2724316" cy="767555"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1130,16 +1306,16 @@
     <col width="3.625" customWidth="1" min="2" max="2"/>
     <col width="7.125" customWidth="1" min="3" max="3"/>
     <col width="65.625" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15.75" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="20.625" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15.75" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12.625" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1246,38 +1422,38 @@
           <t>区　分</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n"/>
+      <c r="C7" s="50" t="n"/>
       <c r="D7" s="15" t="inlineStr">
         <is>
           <t>献立</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="16" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="16" t="n"/>
-      <c r="N7" s="14" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="51" t="n"/>
+      <c r="H7" s="51" t="n"/>
+      <c r="I7" s="51" t="n"/>
+      <c r="J7" s="51" t="n"/>
+      <c r="K7" s="51" t="n"/>
+      <c r="L7" s="51" t="n"/>
+      <c r="M7" s="51" t="n"/>
+      <c r="N7" s="50" t="n"/>
     </row>
     <row r="8" ht="23" customHeight="1">
-      <c r="A8" s="17" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
-      <c r="H8" s="18" t="n"/>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="18" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="18" t="n"/>
-      <c r="N8" s="19" t="n"/>
+      <c r="A8" s="52" t="n"/>
+      <c r="B8" s="53" t="n"/>
+      <c r="C8" s="54" t="n"/>
+      <c r="D8" s="55" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="56" t="n"/>
+      <c r="G8" s="56" t="n"/>
+      <c r="H8" s="56" t="n"/>
+      <c r="I8" s="56" t="n"/>
+      <c r="J8" s="56" t="n"/>
+      <c r="K8" s="56" t="n"/>
+      <c r="L8" s="56" t="n"/>
+      <c r="M8" s="56" t="n"/>
+      <c r="N8" s="54" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
@@ -1308,8 +1484,8 @@
       <c r="N9" s="26" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="27" t="n"/>
-      <c r="B10" s="28" t="n"/>
+      <c r="A10" s="57" t="n"/>
+      <c r="B10" s="58" t="n"/>
       <c r="C10" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1328,7 +1504,7 @@
       <c r="N10" s="33" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="34" t="n"/>
+      <c r="A11" s="57" t="n"/>
       <c r="B11" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -1352,8 +1528,8 @@
       <c r="N11" s="40" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="27" t="n"/>
-      <c r="B12" s="28" t="n"/>
+      <c r="A12" s="57" t="n"/>
+      <c r="B12" s="59" t="n"/>
       <c r="C12" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1372,8 +1548,8 @@
       <c r="N12" s="33" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="41" t="n"/>
-      <c r="B13" s="28" t="n"/>
+      <c r="A13" s="57" t="n"/>
+      <c r="B13" s="58" t="n"/>
       <c r="C13" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1392,7 +1568,7 @@
       <c r="N13" s="33" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="42" t="n"/>
+      <c r="A14" s="57" t="n"/>
       <c r="B14" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -1416,8 +1592,8 @@
       <c r="N14" s="40" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="27" t="n"/>
-      <c r="B15" s="28" t="n"/>
+      <c r="A15" s="57" t="n"/>
+      <c r="B15" s="59" t="n"/>
       <c r="C15" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1436,8 +1612,8 @@
       <c r="N15" s="33" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="n"/>
+      <c r="A16" s="60" t="n"/>
+      <c r="B16" s="58" t="n"/>
       <c r="C16" s="45" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1484,8 +1660,8 @@
       <c r="N17" s="26" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="27" t="n"/>
-      <c r="B18" s="28" t="n"/>
+      <c r="A18" s="57" t="n"/>
+      <c r="B18" s="58" t="n"/>
       <c r="C18" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1504,7 +1680,7 @@
       <c r="N18" s="33" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="34" t="n"/>
+      <c r="A19" s="57" t="n"/>
       <c r="B19" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -1528,8 +1704,8 @@
       <c r="N19" s="40" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="27" t="n"/>
-      <c r="B20" s="28" t="n"/>
+      <c r="A20" s="57" t="n"/>
+      <c r="B20" s="59" t="n"/>
       <c r="C20" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1548,8 +1724,8 @@
       <c r="N20" s="33" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="n"/>
-      <c r="B21" s="28" t="n"/>
+      <c r="A21" s="57" t="n"/>
+      <c r="B21" s="58" t="n"/>
       <c r="C21" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1568,7 +1744,7 @@
       <c r="N21" s="33" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="42" t="n"/>
+      <c r="A22" s="57" t="n"/>
       <c r="B22" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -1592,8 +1768,8 @@
       <c r="N22" s="40" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="27" t="n"/>
-      <c r="B23" s="28" t="n"/>
+      <c r="A23" s="57" t="n"/>
+      <c r="B23" s="59" t="n"/>
       <c r="C23" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1612,8 +1788,8 @@
       <c r="N23" s="33" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="43" t="n"/>
-      <c r="B24" s="44" t="n"/>
+      <c r="A24" s="60" t="n"/>
+      <c r="B24" s="58" t="n"/>
       <c r="C24" s="45" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1660,8 +1836,8 @@
       <c r="N25" s="26" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="28" t="n"/>
+      <c r="A26" s="57" t="n"/>
+      <c r="B26" s="58" t="n"/>
       <c r="C26" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1680,7 +1856,7 @@
       <c r="N26" s="33" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="34" t="n"/>
+      <c r="A27" s="57" t="n"/>
       <c r="B27" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -1704,8 +1880,8 @@
       <c r="N27" s="40" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="27" t="n"/>
-      <c r="B28" s="28" t="n"/>
+      <c r="A28" s="57" t="n"/>
+      <c r="B28" s="59" t="n"/>
       <c r="C28" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1724,8 +1900,8 @@
       <c r="N28" s="33" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="41" t="n"/>
-      <c r="B29" s="28" t="n"/>
+      <c r="A29" s="57" t="n"/>
+      <c r="B29" s="58" t="n"/>
       <c r="C29" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1744,7 +1920,7 @@
       <c r="N29" s="33" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="42" t="n"/>
+      <c r="A30" s="57" t="n"/>
       <c r="B30" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -1768,8 +1944,8 @@
       <c r="N30" s="40" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="27" t="n"/>
-      <c r="B31" s="28" t="n"/>
+      <c r="A31" s="57" t="n"/>
+      <c r="B31" s="59" t="n"/>
       <c r="C31" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1788,8 +1964,8 @@
       <c r="N31" s="33" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="43" t="n"/>
-      <c r="B32" s="44" t="n"/>
+      <c r="A32" s="60" t="n"/>
+      <c r="B32" s="58" t="n"/>
       <c r="C32" s="45" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1836,8 +2012,8 @@
       <c r="N33" s="26" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="27" t="n"/>
-      <c r="B34" s="28" t="n"/>
+      <c r="A34" s="57" t="n"/>
+      <c r="B34" s="58" t="n"/>
       <c r="C34" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1856,7 +2032,7 @@
       <c r="N34" s="33" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="34" t="n"/>
+      <c r="A35" s="57" t="n"/>
       <c r="B35" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -1880,8 +2056,8 @@
       <c r="N35" s="40" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="28" t="n"/>
+      <c r="A36" s="57" t="n"/>
+      <c r="B36" s="59" t="n"/>
       <c r="C36" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1900,8 +2076,8 @@
       <c r="N36" s="33" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="41" t="n"/>
-      <c r="B37" s="28" t="n"/>
+      <c r="A37" s="57" t="n"/>
+      <c r="B37" s="58" t="n"/>
       <c r="C37" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -1920,7 +2096,7 @@
       <c r="N37" s="33" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="42" t="n"/>
+      <c r="A38" s="57" t="n"/>
       <c r="B38" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -1944,8 +2120,8 @@
       <c r="N38" s="40" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="27" t="n"/>
-      <c r="B39" s="28" t="n"/>
+      <c r="A39" s="57" t="n"/>
+      <c r="B39" s="59" t="n"/>
       <c r="C39" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -1964,8 +2140,8 @@
       <c r="N39" s="33" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="43" t="n"/>
-      <c r="B40" s="44" t="n"/>
+      <c r="A40" s="60" t="n"/>
+      <c r="B40" s="58" t="n"/>
       <c r="C40" s="45" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2012,8 +2188,8 @@
       <c r="N41" s="26" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="27" t="n"/>
-      <c r="B42" s="28" t="n"/>
+      <c r="A42" s="57" t="n"/>
+      <c r="B42" s="58" t="n"/>
       <c r="C42" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2032,7 +2208,7 @@
       <c r="N42" s="33" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="34" t="n"/>
+      <c r="A43" s="57" t="n"/>
       <c r="B43" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -2056,8 +2232,8 @@
       <c r="N43" s="40" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="27" t="n"/>
-      <c r="B44" s="28" t="n"/>
+      <c r="A44" s="57" t="n"/>
+      <c r="B44" s="59" t="n"/>
       <c r="C44" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -2076,8 +2252,8 @@
       <c r="N44" s="33" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="41" t="n"/>
-      <c r="B45" s="28" t="n"/>
+      <c r="A45" s="57" t="n"/>
+      <c r="B45" s="58" t="n"/>
       <c r="C45" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2096,7 +2272,7 @@
       <c r="N45" s="33" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="42" t="n"/>
+      <c r="A46" s="57" t="n"/>
       <c r="B46" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -2120,8 +2296,8 @@
       <c r="N46" s="40" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="27" t="n"/>
-      <c r="B47" s="28" t="n"/>
+      <c r="A47" s="57" t="n"/>
+      <c r="B47" s="59" t="n"/>
       <c r="C47" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -2140,8 +2316,8 @@
       <c r="N47" s="33" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="43" t="n"/>
-      <c r="B48" s="44" t="n"/>
+      <c r="A48" s="60" t="n"/>
+      <c r="B48" s="58" t="n"/>
       <c r="C48" s="45" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2188,8 +2364,8 @@
       <c r="N49" s="26" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="27" t="n"/>
-      <c r="B50" s="28" t="n"/>
+      <c r="A50" s="57" t="n"/>
+      <c r="B50" s="58" t="n"/>
       <c r="C50" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2208,7 +2384,7 @@
       <c r="N50" s="33" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="34" t="n"/>
+      <c r="A51" s="57" t="n"/>
       <c r="B51" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -2232,8 +2408,8 @@
       <c r="N51" s="40" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="27" t="n"/>
-      <c r="B52" s="28" t="n"/>
+      <c r="A52" s="57" t="n"/>
+      <c r="B52" s="59" t="n"/>
       <c r="C52" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -2252,8 +2428,8 @@
       <c r="N52" s="33" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="41" t="n"/>
-      <c r="B53" s="28" t="n"/>
+      <c r="A53" s="57" t="n"/>
+      <c r="B53" s="58" t="n"/>
       <c r="C53" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2272,7 +2448,7 @@
       <c r="N53" s="33" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="42" t="n"/>
+      <c r="A54" s="57" t="n"/>
       <c r="B54" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -2296,8 +2472,8 @@
       <c r="N54" s="40" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="27" t="n"/>
-      <c r="B55" s="28" t="n"/>
+      <c r="A55" s="57" t="n"/>
+      <c r="B55" s="59" t="n"/>
       <c r="C55" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -2316,8 +2492,8 @@
       <c r="N55" s="33" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="43" t="n"/>
-      <c r="B56" s="44" t="n"/>
+      <c r="A56" s="60" t="n"/>
+      <c r="B56" s="58" t="n"/>
       <c r="C56" s="45" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2364,8 +2540,8 @@
       <c r="N57" s="26" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="27" t="n"/>
-      <c r="B58" s="28" t="n"/>
+      <c r="A58" s="57" t="n"/>
+      <c r="B58" s="58" t="n"/>
       <c r="C58" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2384,7 +2560,7 @@
       <c r="N58" s="33" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="34" t="n"/>
+      <c r="A59" s="57" t="n"/>
       <c r="B59" s="35" t="inlineStr">
         <is>
           <t>昼</t>
@@ -2408,8 +2584,8 @@
       <c r="N59" s="40" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
-      <c r="A60" s="27" t="n"/>
-      <c r="B60" s="28" t="n"/>
+      <c r="A60" s="57" t="n"/>
+      <c r="B60" s="59" t="n"/>
       <c r="C60" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -2428,8 +2604,8 @@
       <c r="N60" s="33" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="41" t="n"/>
-      <c r="B61" s="28" t="n"/>
+      <c r="A61" s="57" t="n"/>
+      <c r="B61" s="58" t="n"/>
       <c r="C61" s="29" t="inlineStr">
         <is>
           <t>副②</t>
@@ -2448,7 +2624,7 @@
       <c r="N61" s="33" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="42" t="n"/>
+      <c r="A62" s="57" t="n"/>
       <c r="B62" s="35" t="inlineStr">
         <is>
           <t>夕</t>
@@ -2472,8 +2648,8 @@
       <c r="N62" s="40" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="27" t="n"/>
-      <c r="B63" s="28" t="n"/>
+      <c r="A63" s="57" t="n"/>
+      <c r="B63" s="59" t="n"/>
       <c r="C63" s="29" t="inlineStr">
         <is>
           <t>副①</t>
@@ -2492,8 +2668,8 @@
       <c r="N63" s="33" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="43" t="n"/>
-      <c r="B64" s="44" t="n"/>
+      <c r="A64" s="60" t="n"/>
+      <c r="B64" s="58" t="n"/>
       <c r="C64" s="45" t="inlineStr">
         <is>
           <t>副②</t>

</xml_diff>

<commit_message>
Fix generated facility template pipeline
</commit_message>
<xml_diff>
--- a/backend/src/data/order_form_master_templates/master_layout_template.xlsx
+++ b/backend/src/data/order_form_master_templates/master_layout_template.xlsx
@@ -40,7 +40,7 @@
     <definedName name="WkMonthNum" localSheetId="0">MONTH(DATEVALUE(#REF!&amp;"/1"))</definedName>
     <definedName name="WkMonthView" localSheetId="0">#REF!</definedName>
     <definedName name="WkWeek" localSheetId="0">LEFT(RIGHT(#REF!,3),1)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'master_layout'!$A$1:$L$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'master_layout'!$A$1:$L$69</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1792,7 +1792,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2450,6 +2450,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="103" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="104" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -2936,11 +2938,6 @@
           <t>FAX送信先：050-3092-0899</t>
         </is>
       </c>
-      <c r="H2" s="194" t="n"/>
-      <c r="I2" s="194" t="n"/>
-      <c r="J2" s="194" t="n"/>
-      <c r="K2" s="194" t="n"/>
-      <c r="L2" s="194" t="n"/>
     </row>
     <row r="3" ht="35.85" customHeight="1" s="193" thickBot="1">
       <c r="A3" s="179" t="inlineStr">
@@ -2948,54 +2945,38 @@
           <t>施設名ご記入お願いします。</t>
         </is>
       </c>
-      <c r="E3" s="194" t="n"/>
       <c r="F3" s="197" t="n"/>
       <c r="G3" s="198" t="inlineStr">
         <is>
           <t>締切日4月10日まで</t>
         </is>
       </c>
-      <c r="H3" s="194" t="n"/>
-      <c r="I3" s="194" t="n"/>
-      <c r="J3" s="194" t="n"/>
-      <c r="K3" s="194" t="n"/>
-      <c r="L3" s="194" t="n"/>
     </row>
     <row r="4" ht="35.85" customHeight="1" s="193">
       <c r="A4" s="199" t="n"/>
       <c r="B4" s="200" t="n"/>
       <c r="C4" s="200" t="n"/>
       <c r="D4" s="200" t="n"/>
-      <c r="E4" s="194" t="n"/>
+      <c r="E4" s="241" t="n"/>
       <c r="F4" s="197" t="n"/>
       <c r="G4" s="201" t="inlineStr">
         <is>
           <t>※ご希望メニューに食数をご記入ください。</t>
         </is>
       </c>
-      <c r="H4" s="194" t="n"/>
-      <c r="I4" s="194" t="n"/>
-      <c r="J4" s="194" t="n"/>
-      <c r="K4" s="194" t="n"/>
-      <c r="L4" s="194" t="n"/>
     </row>
     <row r="5" ht="35.85" customHeight="1" s="193" thickBot="1">
       <c r="A5" s="202" t="n"/>
       <c r="B5" s="203" t="n"/>
       <c r="C5" s="203" t="n"/>
       <c r="D5" s="203" t="n"/>
-      <c r="E5" s="194" t="n"/>
+      <c r="E5" s="242" t="n"/>
       <c r="F5" s="197" t="n"/>
       <c r="G5" s="201" t="inlineStr">
         <is>
           <t>※禁止食材は対象食種に〇をつけ、禁食欄に数字を入れてください。</t>
         </is>
       </c>
-      <c r="H5" s="194" t="n"/>
-      <c r="I5" s="194" t="n"/>
-      <c r="J5" s="194" t="n"/>
-      <c r="K5" s="194" t="n"/>
-      <c r="L5" s="194" t="n"/>
     </row>
     <row r="6" ht="35.65" customHeight="1" s="193" thickBot="1">
       <c r="A6" s="91" t="n"/>
@@ -3009,11 +2990,6 @@
           <t>※副菜の禁食対応はご相談ください。</t>
         </is>
       </c>
-      <c r="H6" s="194" t="n"/>
-      <c r="I6" s="194" t="n"/>
-      <c r="J6" s="194" t="n"/>
-      <c r="K6" s="194" t="n"/>
-      <c r="L6" s="194" t="n"/>
     </row>
     <row r="7" ht="18.75" customHeight="1" s="193">
       <c r="A7" s="156" t="inlineStr">
@@ -4186,8 +4162,8 @@
   <mergeCells count="105">
     <mergeCell ref="B53:B55"/>
     <mergeCell ref="E18:L18"/>
+    <mergeCell ref="E58:L58"/>
     <mergeCell ref="E43:L43"/>
-    <mergeCell ref="E58:L58"/>
     <mergeCell ref="B43:B44"/>
     <mergeCell ref="G6:L6"/>
     <mergeCell ref="E33:L33"/>
@@ -4307,214 +4283,214 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>layout_role</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>master_layout</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>source_workbook</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>/Users/mmorinag/Sawa/2025.12/input_example/発注書/共通　2604.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>source_sheet</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>4月26日～4月30日</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>body_start_row</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>body_end_row</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>66</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>days_per_page</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>header_top_row</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>header_group_bottom_row</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>header_leaf_top_row</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>header_bottom_row</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>fixed_date_cols</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>fixed_daypart_cols</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>B:C</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>fixed_menu_cols</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>generated_columns_area_cols</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>E:L</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>fixed_width_policy</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>A:D copied from source workbook exactly; generated columns total equals source E:L</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>two_level_header_rule</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>merge contiguous identical header_group values only</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>remarks_position</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>generated after quantity columns; absorbs remaining generated width when needed</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>source_policy</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>derived from common 2026-04 source workbook layout with variable values cleared</t>
         </is>

</xml_diff>